<commit_message>
Delmtr_Cd holds the delimiter character itself
The column takes the one delimiter character (|, ",", *, ; ...), \t for a tab; empty = comma.
The word codes PIPE / COMMA / TAB / SEMICOLON are no longer accepted: validate-config reports
them (DELIMITER) and FILE_CHECK reports a CONFIG finding. Example workbooks, guides and the
design note updated; Glue wheel 0.3.14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -4227,7 +4227,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>|</t>
         </is>
       </c>
       <c r="G5" s="10" t="n">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>|</t>
         </is>
       </c>
       <c r="G6" s="10" t="n">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>|</t>
         </is>
       </c>
       <c r="G7" s="10" t="n">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>|</t>
         </is>
       </c>
       <c r="G8" s="10" t="n">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>|</t>
         </is>
       </c>
       <c r="G9" s="10" t="n">

</xml_diff>

<commit_message>
COLUMN_VALUES check for every record; control characters; faster content checks
- FILE_CHECK: optional COLUMN_VALUES check (ALL, or LENGTH / NUMBER / REQUIRED): every value of
  every data row against its target staging column, from the column definitions the database
  reports. All offending records go to the error file before the load.
- CHARACTER_SET also reports control characters (tab excepted).
- Both checks test a whole row cheaply first and look at single values only in a row that fails:
  about 270,000 rows per second for a 25-column file with every check on.
- Glue wheel 0.3.18; guides, design note and the CMSUNIV sample updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -5783,13 +5783,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
@@ -5798,10 +5798,10 @@
     <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="96" customHeight="1">
+    <row r="1" ht="128" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Which content checks FILE_CHECK applies. The three '*' rows are the defaults for every ODAG3 source: header names, H / D / T record types and the trailer layout. The two rows with Active_Ind = 0 switch the record types off for the internal sources, whose files have no record type (their trailer check does not apply either, because Src_File_Has_Trlr_Ind = 0). The header names here are the table's column names, as a placeholder: put the real header line of the ODAG3 file. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Which content checks FILE_CHECK applies. CHARACTER_SET and COLUMN_VALUES apply to every table of the project: every line must be Latin text and every value must fit its target column (length, number, NOT NULL); all offending records go to the error file. The three ODAG3 '*' rows are the defaults for every ODAG3 source: header names, H / D / T record types and the trailer layout. The two rows with Active_Ind = 0 switch the record types off for the internal sources, whose files have no record type (their trailer check does not apply either, because Src_File_Has_Trlr_Ind = 0). The header names here are the table's column names, as a placeholder: put the real header line of the ODAG3 file. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -6067,22 +6067,26 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>ODAG3</t>
+          <t>*</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>*</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>RECORD_TYPE</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n"/>
+          <t>CHARACTER_SET</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>latin-1</t>
+        </is>
+      </c>
       <c r="F8" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -6113,39 +6117,135 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>COLUMN_VALUES</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
           <t>ODAG3</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>RECORD_TYPE</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>RECORD_TYPE</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n">
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>

</xml_diff>

<commit_message>
Staging always cleared by run type; Include_Ind on file checks
- ComplianceSourceFileConfig.Stg_Cleanup_Cd is removed: before a load every staging row of the
  file's run type is deleted (a staging table without a run type column is cleared by batch).
- ComplianceFileCheckConfig.Include_Ind says whether a check applies to (1) or is excluded from
  (0) the files a row covers. Active_Ind = 0 now only means the row is ignored. Per check the
  most specific active row wins, whether it includes or excludes: table and source, then table,
  then source, then '*'. The same reading of Active_Ind applies to ComplianceTargetColumnConfig.
- Glue wheel 0.3.20; guides, design note and the CMSUNIV sample updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -4493,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4511,18 +4511,17 @@
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="32" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="32" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="96" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>One row per source: what the file looks like and where it loads. Cfg_ID is generated: leave it out of the INSERT. FDR files have a header and a trailer; internal files have a header only. Delmtr_Cd is the delimiter character itself. All FDR files arrive in one folder and all internal files in another; the name template tells them apart. Stg_Cleanup_Cd = RUN_TYPE clears the staging rows of the file's run type before each load. $env / $ENV resolve to the environment of the run. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>One row per source: what the file looks like and where it loads. Cfg_ID is generated: leave it out of the INSERT. FDR files have a header and a trailer; internal files have a header only. Delmtr_Cd is the delimiter character itself. All FDR files arrive in one folder and all internal files in another; the name template tells them apart. Before each load the staging rows of the file's run type are removed. $env / $ENV resolve to the environment of the run. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -4604,30 +4603,25 @@
       </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
-          <t>Stg_Cleanup_Cd</t>
+          <t>Active_Ind</t>
         </is>
       </c>
       <c r="Q3" s="8" t="inlineStr">
         <is>
-          <t>Active_Ind</t>
+          <t>Created_Dtts</t>
         </is>
       </c>
       <c r="R3" s="8" t="inlineStr">
         <is>
-          <t>Created_Dtts</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="S3" s="8" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Updated_Dtts</t>
         </is>
       </c>
       <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_Dtts</t>
-        </is>
-      </c>
-      <c r="U3" s="8" t="inlineStr">
         <is>
           <t>Updated_By</t>
         </is>
@@ -4711,30 +4705,25 @@
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10) DEFAULT 'BATCH' NOT NULL</t>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
       <c r="R4" s="9" t="inlineStr">
         <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr">
+        <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="S4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
       <c r="T4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="U4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
@@ -4810,30 +4799,25 @@
           <t>22</t>
         </is>
       </c>
-      <c r="P5" s="13" t="inlineStr">
-        <is>
-          <t>RUN_TYPE</t>
-        </is>
-      </c>
-      <c r="Q5" s="10" t="n">
+      <c r="P5" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="Q5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
       <c r="R5" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="S5" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="T5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="U5" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -4909,30 +4893,25 @@
           <t>22</t>
         </is>
       </c>
-      <c r="P6" s="13" t="inlineStr">
-        <is>
-          <t>RUN_TYPE</t>
-        </is>
-      </c>
-      <c r="Q6" s="10" t="n">
+      <c r="P6" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="Q6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="S6" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="T6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="U6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5008,30 +4987,25 @@
           <t>22</t>
         </is>
       </c>
-      <c r="P7" s="13" t="inlineStr">
-        <is>
-          <t>RUN_TYPE</t>
-        </is>
-      </c>
-      <c r="Q7" s="10" t="n">
+      <c r="P7" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="Q7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
       <c r="R7" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="S7" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="T7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="U7" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5107,30 +5081,25 @@
           <t>22</t>
         </is>
       </c>
-      <c r="P8" s="13" t="inlineStr">
-        <is>
-          <t>RUN_TYPE</t>
-        </is>
-      </c>
-      <c r="Q8" s="10" t="n">
+      <c r="P8" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="Q8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="S8" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="T8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="U8" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5206,30 +5175,25 @@
           <t>22</t>
         </is>
       </c>
-      <c r="P9" s="13" t="inlineStr">
-        <is>
-          <t>RUN_TYPE</t>
-        </is>
-      </c>
-      <c r="Q9" s="10" t="n">
+      <c r="P9" s="10" t="n">
         <v>1</v>
       </c>
+      <c r="Q9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
       <c r="R9" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="S9" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="T9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="U9" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5237,7 +5201,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:T1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5783,7 +5747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5791,17 +5755,18 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="128" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Which content checks FILE_CHECK applies. CHARACTER_SET and COLUMN_VALUES apply to every table of the project: every line must be Latin text and every value must fit its target column (length, number, NOT NULL); all offending records go to the error file. The three ODAG3 '*' rows are the defaults for every ODAG3 source: header names, H / D / T record types and the trailer layout. The two rows with Active_Ind = 0 switch the record types off for the internal sources, whose files have no record type (their trailer check does not apply either, because Src_File_Has_Trlr_Ind = 0). The header names here are the table's column names, as a placeholder: put the real header line of the ODAG3 file. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Which content checks FILE_CHECK applies. CHARACTER_SET and COLUMN_VALUES apply to every table of the project: every line must be Latin text and every value must fit its target column (length, number, NOT NULL); all offending records go to the error file. The three ODAG3 '*' rows are the defaults for every ODAG3 source: header names, H / D / T record types and the trailer layout. The two rows with Include_Ind = 0 exclude the internal sources from the record type check, since their files have none (their trailer check does not apply either, because Src_File_Has_Trlr_Ind = 0). The header names here are the table's column names, as a placeholder: put the real header line of the ODAG3 file. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -5833,25 +5798,30 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
+          <t>Include_Ind</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
           <t>Active_Ind</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Created_Dtts</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Created_By</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Updated_Dtts</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>Updated_By</t>
         </is>
@@ -5890,20 +5860,25 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
@@ -5935,25 +5910,28 @@
           <t>MemberFirstName|MemberLastName|MemberID|ContractID|PlanBenefitPackage|FirstTierDownstreamandRelatedEntity|AuthorizationorClaimNumber|Datetherequestwasreceived|AORReceiptDate|WaiverofLiabilityReceiptDate|WasItaCleanClaim|WasTheRequestProcessedasanODorRecon|RequestDetermination|DateofDetermination|DateClaimReconsiderationwasPaid|DateWrittenNotificationprovidedToMember|DateWrittenNotificationProvidedtoProvider|DateForwardedtoIRE|Whomadetherequest|Issuedescriptionandtypeofservice|WasTheInitOrgDetReqtDeniedForLackOfMediNecessity|ExRMNumber|SourceUnique_ID|Filler2|Filler3</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G5" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5985,25 +5963,28 @@
           <t>H,D,T</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G6" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6035,25 +6016,28 @@
           <t>RECORD_TYPE,FILE_NAME,TOTAL_ROW_COUNT,TIMESTAMP</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G7" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6085,25 +6069,28 @@
           <t>latin-1</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G8" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6135,25 +6122,28 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G9" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6184,22 +6174,25 @@
       <c r="F10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G10" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6230,22 +6223,25 @@
       <c r="F11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
+      <c r="G11" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6253,7 +6249,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Target columns: CONSTANT, LOAD_DATE and SQL values
ComplianceTargetColumnConfig.Value_Txt with three more Value_Cd:
- CONSTANT: the literal in Value_Txt on every row.
- LOAD_DATE: the date of the load (text YYYY-MM-DD in a character column).
- SQL: Value_Txt is a single SELECT returning one value, run once per load before staging,
  with the load's values as bound {name} parameters (PostgreSQL runs it read-only). A statement
  that fails or does not return exactly one value stops the load of that file.
validate-config checks the rows without running the statements. Glue wheel 0.3.21; guides,
design note and the CMSUNIV sample workbook and SQL file updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -5213,24 +5213,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="80" customHeight="1">
+    <row r="1" ht="112" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Which columns of the staging and core tables the framework fills. Every other column of the staging table is a column of the file, in table order (the 25 ODAG3 columns here). The '*' rows apply to every CMSUNIV table; the row ID is one row per table. Btch_ID needs no row. Current_Ind and End_Dtts are core-table columns: an earlier load of a batch is flagged 0, the new rows are added as 1, so core always holds the data. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Which columns of the staging and core tables the framework fills. Every other column of the staging table is a column of the file, in table order (the 25 ODAG3 columns here). The '*' rows apply to every CMSUNIV table; the row ID is one row per table. Btch_ID needs no row. Current_Ind and End_Dtts are core-table columns: an earlier load of a batch is flagged 0, the new rows are added as 1, so core always holds the data. Value_Txt is only filled for two more codes these tables do not need: CONSTANT (a fixed value such as Y) and SQL (a SELECT returning one value, for example an audit ID from another table). Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -5257,25 +5258,30 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
+          <t>Value_Txt</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
           <t>Active_Ind</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Created_Dtts</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Created_By</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Updated_Dtts</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Updated_By</t>
         </is>
@@ -5304,25 +5310,30 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
+          <t>VARCHAR(8000)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
           <t>SMALLINT DEFAULT 1 NOT NULL</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
@@ -5349,25 +5360,26 @@
           <t>LOAD_TIMESTAMP</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5394,25 +5406,26 @@
           <t>VERSION</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5439,25 +5452,26 @@
           <t>RUN_TYPE</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5484,25 +5498,26 @@
           <t>FILE_NAME</t>
         </is>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5529,25 +5544,26 @@
           <t>SOURCE_ID</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5574,25 +5590,26 @@
           <t>LOAD_TIMESTAMP</t>
         </is>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5619,25 +5636,26 @@
           <t>CURRENT_FLAG</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5664,25 +5682,26 @@
           <t>END_TIMESTAMP</t>
         </is>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5709,25 +5728,26 @@
           <t>ROW_SEQUENCE</t>
         </is>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5735,7 +5755,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Core load: delete the batch's rows by Btch_ID, then insert
- The core table needs no current-flag or end-date column; CURRENT_FLAG
  and END_TIMESTAMP stay accepted as optional value codes.
- Sample workbook and INSERT scripts regenerated without those rows.
- Version 0.3.24.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -574,7 +574,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Staging and core tables ODAG_DE_TABLE3_2022 in the existing layout: row ID, the 25 file columns, then StagingCreateDate, Btch_ID, Universe_Vrsn, Run_Ty, FileName, Src_Data_Key, Load_Dtts; the core table also has Current_Ind and End_Dtts.</t>
+          <t>Staging and core tables ODAG_DE_TABLE3_2022 in the existing layout: row ID, the 25 file columns, then StagingCreateDate, Btch_ID, Universe_Vrsn, Run_Ty, FileName, Src_Data_Key, Load_Dtts, in both tables.</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5231,7 +5231,7 @@
     <row r="1" ht="112" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Which columns of the staging and core tables the framework fills. Every other column of the staging table is a column of the file, in table order (the 25 ODAG3 columns here). The '*' rows apply to every CMSUNIV table; the row ID is one row per table. Btch_ID needs no row. Current_Ind and End_Dtts are core-table columns: an earlier load of a batch is flagged 0, the new rows are added as 1, so core always holds the data. Value_Txt is only filled for two more codes these tables do not need: CONSTANT (a fixed value such as Y) and SQL (a SELECT returning one value, for example an audit ID from another table). Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Which columns of the staging and core tables the framework fills. Every other column of the staging table is a column of the file, in table order (the 25 ODAG3 columns here). The '*' rows apply to every CMSUNIV table; the row ID is one row per table. Btch_ID needs no row. When a file is loaded for a batch that already has rows in the core table, those rows are deleted by Btch_ID and the new rows are inserted. Value_Txt is only filled for two more codes these tables do not need: CONSTANT (a fixed value such as Y) and SQL (a SELECT returning one value, for example an audit ID from another table). Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -5623,17 +5623,17 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>ODAG3</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Current_Ind</t>
+          <t>ODAG_DE_Table3_2022_ID</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>CURRENT_FLAG</t>
+          <t>ROW_SEQUENCE</t>
         </is>
       </c>
       <c r="E11" s="10" t="n"/>
@@ -5656,98 +5656,6 @@
         </is>
       </c>
       <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>End_Dtts</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>END_TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>ODAG_DE_Table3_2022_ID</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>ROW_SEQUENCE</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>

</xml_diff>

<commit_message>
Batch status names, step report in the log, scope by project / table group / table / run type
- Req_Stat: PROMOTED -> SOURCE_DATA_READY, CARRIED_FORWARD ->
  SOURCE_DATA_CARRY_FORWARD, COMPLETED -> REQUEST_COMPLETE. A file with no
  data rows is the source's delivery: SOURCE_DATA_READY_NO_DATA (Resolution_Ty
  NO_DATA), closed as DATA_NOT_PROVIDED; Allow_Zero_Rcd_Ind no longer used.
- Every step ends with one indented report in the log (per file for FILE_LOAD
  and FILE_CHECK: status, batch, batch status, rows, reason, detail, error
  log); progress lines without file data; one-line events; SMB chatter off.
- Every step takes project, optionally table_group or table, optionally
  run_type. Table groups in the optional ComplianceTable, read only when a
  run names one. Triggered DAGs inherit the scope; Glue takes table_group.
- Version 0.3.33.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -9,18 +9,19 @@
   <sheets>
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ComplianceProject" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ComplianceSourceSystem" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ComplianceRunType" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ComplianceDataSetSourceXwalk" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ComplianceSourceFileConfig" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ComplianceTargetColumnConfig" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ComplianceFileCheckConfig" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ComplianceRuleBinding" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="ComplianceRequestInTake" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ComplianceBatchOverride" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Airflow Variables" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sample files" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Expected batches" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="ComplianceTable" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ComplianceSourceSystem" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ComplianceRunType" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ComplianceDataSetSourceXwalk" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ComplianceSourceFileConfig" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ComplianceTargetColumnConfig" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ComplianceFileCheckConfig" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ComplianceRuleBinding" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ComplianceRequestInTake" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ComplianceBatchOverride" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Airflow Variables" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Sample files" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Expected batches" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -734,6 +735,212 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Optional: only when FILE_RULES should run GRE rules on loaded files. '*' = every source / run type. The rule group and variant are examples and must exist in the GRE. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Src_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Run_Ty</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Gre_Rule_Group</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Gre_Rule_Variant</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(20) DEFAULT '*' NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) NOT NULL</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_ODAG3</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>DEFAULT</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1028,7 +1235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1282,7 +1489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1572,7 +1779,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2103,7 +2310,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3011,6 +3218,180 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Optional: the table group of each table. Only needed to run a step for a table group (e.g. table_group ODAG for ODAG1 to ODAG5); without rows here every step works per project or per table as before. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Grp_Cd</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Desc</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(200)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG table 3</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3323,7 +3704,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3626,7 +4007,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4487,7 +4868,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5207,7 +5588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5669,7 +6050,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6181,210 +6562,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="48" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Optional: only when FILE_RULES should run GRE rules on loaded files. '*' = every source / run type. The rule group and variant are examples and must exist in the GRE. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Project_Cd</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Table_Nm</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Src_ID</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Run_Ty</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Gre_Rule_Group</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Gre_Rule_Variant</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Active_Ind</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Created_Dtts</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Created_By</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_Dtts</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_By</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(63) NOT NULL</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(20) DEFAULT '*' NOT NULL</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) NOT NULL</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) NOT NULL</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV_ODAG3</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>DEFAULT</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Sample metadata: query sources, export config, REOPEN override
- ComplianceSourceQueryConfig: internal source 30 on the same Teradata
  system and 40 on SQL Server (Airflow Connection cms_src_appeals_sqlsrv),
  with their source system and crosswalk rows.
- ComplianceExportConfig for ODAG3, with the export table DDL and an UPDATE
  example for an export procedure.
- REOPEN override example next to the REUSE one.
- Workbook regenerated with the same rows; every statement checked by
  running it and reading the rows back.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -14,14 +14,16 @@
     <sheet name="ComplianceRunType" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="ComplianceDataSetSourceXwalk" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ComplianceSourceFileConfig" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ComplianceTargetColumnConfig" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ComplianceFileCheckConfig" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="ComplianceRuleBinding" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ComplianceRequestInTake" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ComplianceBatchOverride" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Airflow Variables" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Sample files" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Expected batches" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="ComplianceSourceQueryConfig" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ComplianceTargetColumnConfig" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ComplianceExportConfig" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ComplianceFileCheckConfig" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ComplianceRuleBinding" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ComplianceRequestInTake" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ComplianceBatchOverride" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Airflow Variables" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Sample files" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Expected batches" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -735,6 +737,730 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="80" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Optional: the export table of a core table (EXPORT_LOAD). It has the core table's columns (the row ID included) and Btch_ID, plus Exp_Btch_ID for the export batch (another name: Exp_Btch_Col_Nm). Exp_Proc_Nm / Exp_Proc_Parm_Txt: a procedure that does the export instead of the framework's delete and INSERT ... SELECT (an UPDATE example is in cmsuniv_odag3_sample_metadata.sql). Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Exp_Schema_Nm</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Exp_Table_Nm</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Exp_Btch_Col_Nm</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Exp_Proc_Nm</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Exp_Proc_Parm_Txt</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(256)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(1000)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_EXPORT_$ENV_T</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022_EXP</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="128" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Which content checks FILE_CHECK applies. CHARACTER_SET and COLUMN_VALUES apply to every table of the project: every line must be Latin text and every value must fit its target column (length, number, NOT NULL); all offending records go to the error file. The three ODAG3 '*' rows are the defaults for every ODAG3 source: header names, H / D / T record types and the trailer layout. The two rows with Include_Ind = 0 exclude the internal sources from the record type check, since their files have none (their trailer check does not apply either, because Src_File_Has_Trlr_Ind = 0). The header names here are the table's column names, as a placeholder: put the real header line of the ODAG3 file. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Src_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Check_Cd</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Check_Val_Txt</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Include_Ind</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) DEFAULT '*' NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) DEFAULT '*' NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(8000)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>HEADER_NAMES</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>MemberFirstName|MemberLastName|MemberID|ContractID|PlanBenefitPackage|FirstTierDownstreamandRelatedEntity|AuthorizationorClaimNumber|Datetherequestwasreceived|AORReceiptDate|WaiverofLiabilityReceiptDate|WasItaCleanClaim|WasTheRequestProcessedasanODorRecon|RequestDetermination|DateofDetermination|DateClaimReconsiderationwasPaid|DateWrittenNotificationprovidedToMember|DateWrittenNotificationProvidedtoProvider|DateForwardedtoIRE|Whomadetherequest|Issuedescriptionandtypeofservice|WasTheInitOrgDetReqtDeniedForLackOfMediNecessity|ExRMNumber|SourceUnique_ID|Filler2|Filler3</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>RECORD_TYPE</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>H,D,T</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>TRAILER</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>RECORD_TYPE,FILE_NAME,TOTAL_ROW_COUNT,TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>CHARACTER_SET</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>latin-1</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>COLUMN_VALUES</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>RECORD_TYPE</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>RECORD_TYPE</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -935,7 +1661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1235,13 +1961,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1260,10 +1986,10 @@
     <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="80" customHeight="1">
+    <row r="1" ht="96" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Only when a carry-forward is wanted: an approved REUSE override lets an open CMS batch without a file reuse the data of an earlier closed batch of the same table, source and run type. Entered after the batches exist; Btch_ID / Req_ID are those of the batch that will reuse, Reuse_Btch_ID the earlier batch (empty = the latest one). OVERRIDE_DECISIONS applies it. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Only when a carry-forward is wanted: an approved REUSE override lets an open CMS batch without a file reuse the data of an earlier closed batch of the same table, source and run type. Entered after the batches exist; Btch_ID / Req_ID are those of the batch that will reuse, Reuse_Btch_ID the earlier batch (empty = the latest one). OVERRIDE_DECISIONS applies it. REOPEN (second row): opens a closed batch again until new data arrives; applied once by OVERRIDE_DECISIONS. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -1476,6 +2202,72 @@
         </is>
       </c>
       <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>(identity)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>REOPEN</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>(Req_ID of the batch)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>20261019_CMSUNIV_ODAG3_140_CMS_2200_1</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>46326</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>ESI resends corrected data for the closed CMS request</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>approver_id</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:00:00</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -1489,7 +2281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1779,7 +2571,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2310,29 +3102,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
     <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1">
+    <row r="1" ht="64" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>What BATCH_CREATION created from these rows when it ran on Fri 2026-10-16, Mon 2026-10-19, Tue 2026-10-20 and Wed 2026-10-21 (observed, not hand-written). On 10-20 and 10-21 the MNT batches already existed, so only DAILY (and one CMS request) were added.</t>
+          <t>What BATCH_CREATION created from these rows when it ran on Fri 2026-10-16, Mon 2026-10-19, Tue 2026-10-20 and Wed 2026-10-21 (observed, not hand-written). The batches of the query sources (30, 40) get their data from SOURCE_LOAD, not from a file. On 10-20 and 10-21 the MNT batches already existed, so only DAILY (and one CMS request) were added.</t>
         </is>
       </c>
     </row>
@@ -2452,73 +3244,73 @@
     </row>
     <row r="6">
       <c r="A6" s="17" t="n">
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>CMS</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>UMAuth</t>
         </is>
       </c>
       <c r="E6" s="17" t="n">
-        <v>46204</v>
+        <v>46310</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_10_CMS_2200_1</t>
+          <t>20261016_CMSUNIV_ODAG3_30_DAILY_2200_1</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>ComplianceRequestInTake request due that day</t>
+          <t>DAILY is due every day: the previous day</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="n">
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>CMS</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>OptumRx</t>
+          <t>AppealsDB</t>
         </is>
       </c>
       <c r="E7" s="17" t="n">
-        <v>46204</v>
+        <v>46310</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>46295</v>
+        <v>46310</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_130_CMS_2200_1</t>
+          <t>20261016_CMSUNIV_ODAG3_40_DAILY_2200_1</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>ComplianceRequestInTake request due that day</t>
+          <t>DAILY is due every day: the previous day</t>
         </is>
       </c>
     </row>
@@ -2533,12 +3325,12 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>ESI</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="E8" s="17" t="n">
@@ -2549,7 +3341,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_140_CMS_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_10_CMS_2200_1</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -2569,12 +3361,12 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Appeals</t>
+          <t>OptumRx</t>
         </is>
       </c>
       <c r="E9" s="17" t="n">
@@ -2585,7 +3377,7 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_20_CMS_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_130_CMS_2200_1</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -2605,12 +3397,12 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>140</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>MedHOK</t>
+          <t>ESI</t>
         </is>
       </c>
       <c r="E10" s="17" t="n">
@@ -2621,7 +3413,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_51_CMS_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_140_CMS_2200_1</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -2636,33 +3428,33 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>Appeals</t>
         </is>
       </c>
       <c r="E11" s="17" t="n">
-        <v>46313</v>
+        <v>46204</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>46313</v>
+        <v>46295</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_10_DAILY_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_20_CMS_2200_1</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>DAILY is due every day: the previous day</t>
+          <t>ComplianceRequestInTake request due that day</t>
         </is>
       </c>
     </row>
@@ -2672,33 +3464,33 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Appeals</t>
+          <t>UMAuth</t>
         </is>
       </c>
       <c r="E12" s="17" t="n">
-        <v>46313</v>
+        <v>46204</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>46313</v>
+        <v>46295</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_20_DAILY_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_30_CMS_2200_1</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>DAILY is due every day: the previous day</t>
+          <t>ComplianceRequestInTake request due that day</t>
         </is>
       </c>
     </row>
@@ -2708,33 +3500,33 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>AppealsDB</t>
         </is>
       </c>
       <c r="E13" s="17" t="n">
-        <v>46266</v>
+        <v>46204</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>46295</v>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_10_MNT_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_40_CMS_2200_1</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>ComplianceRequestInTake request due that day</t>
         </is>
       </c>
     </row>
@@ -2744,33 +3536,33 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>51</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>OptumRx</t>
+          <t>MedHOK</t>
         </is>
       </c>
       <c r="E14" s="17" t="n">
-        <v>46266</v>
+        <v>46204</v>
       </c>
       <c r="F14" s="17" t="n">
         <v>46295</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_130_MNT_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_51_CMS_2200_1</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>ComplianceRequestInTake request due that day</t>
         </is>
       </c>
     </row>
@@ -2780,33 +3572,33 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>ESI</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="E15" s="17" t="n">
-        <v>46266</v>
+        <v>46313</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>46295</v>
+        <v>46313</v>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_140_MNT_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_10_DAILY_2200_1</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>DAILY is due every day: the previous day</t>
         </is>
       </c>
     </row>
@@ -2816,7 +3608,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -2830,19 +3622,19 @@
         </is>
       </c>
       <c r="E16" s="17" t="n">
-        <v>46266</v>
+        <v>46313</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>46295</v>
+        <v>46313</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_20_MNT_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_20_DAILY_2200_1</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>DAILY is due every day: the previous day</t>
         </is>
       </c>
     </row>
@@ -2852,39 +3644,39 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>MedHOK</t>
+          <t>UMAuth</t>
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>46266</v>
+        <v>46313</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>46295</v>
+        <v>46313</v>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>20261019_CMSUNIV_ODAG3_51_MNT_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_30_DAILY_2200_1</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>DAILY is due every day: the previous day</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
@@ -2893,23 +3685,23 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>AppealsDB</t>
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>20261020_CMSUNIV_ODAG3_10_DAILY_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_40_DAILY_2200_1</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -2920,143 +3712,575 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>MNT</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Appeals</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>46314</v>
+        <v>46266</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>46314</v>
+        <v>46295</v>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>20261020_CMSUNIV_ODAG3_20_DAILY_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_10_MNT_2200_1</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>DAILY is due every day: the previous day</t>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="n">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>CMS</t>
+          <t>MNT</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>ESI</t>
+          <t>OptumRx</t>
         </is>
       </c>
       <c r="E20" s="17" t="n">
-        <v>46113</v>
+        <v>46266</v>
       </c>
       <c r="F20" s="17" t="n">
-        <v>46203</v>
+        <v>46295</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>20261021_CMSUNIV_ODAG3_140_CMS_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_130_MNT_2200_1</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>ComplianceRequestInTake request due that day</t>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="n">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>MNT</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>140</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>ESI</t>
         </is>
       </c>
       <c r="E21" s="17" t="n">
-        <v>46315</v>
+        <v>46266</v>
       </c>
       <c r="F21" s="17" t="n">
-        <v>46315</v>
+        <v>46295</v>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>20261021_CMSUNIV_ODAG3_10_DAILY_2200_1</t>
+          <t>20261019_CMSUNIV_ODAG3_140_MNT_2200_1</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>DAILY is due every day: the previous day</t>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Appeals</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>20261019_CMSUNIV_ODAG3_20_MNT_2200_1</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>UMAuth</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>20261019_CMSUNIV_ODAG3_30_MNT_2200_1</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>AppealsDB</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>20261019_CMSUNIV_ODAG3_40_MNT_2200_1</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>MedHOK</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>20261019_CMSUNIV_ODAG3_51_MNT_2200_1</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Claims</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>20261020_CMSUNIV_ODAG3_10_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Appeals</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>20261020_CMSUNIV_ODAG3_20_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>UMAuth</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>20261020_CMSUNIV_ODAG3_30_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>AppealsDB</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>20261020_CMSUNIV_ODAG3_40_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
         <v>46316</v>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>ESI</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="n">
+        <v>46113</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>46203</v>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>20261021_CMSUNIV_ODAG3_140_CMS_2200_1</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>ComplianceRequestInTake request due that day</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>DAILY</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Claims</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>20261021_CMSUNIV_ODAG3_10_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n">
+      <c r="E32" s="17" t="n">
         <v>46315</v>
       </c>
-      <c r="F22" s="17" t="n">
+      <c r="F32" s="17" t="n">
         <v>46315</v>
       </c>
-      <c r="G22" s="11" t="inlineStr">
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>20261021_CMSUNIV_ODAG3_20_DAILY_2200_1</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>UMAuth</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>20261021_CMSUNIV_ODAG3_30_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>DAILY is due every day: the previous day</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>AppealsDB</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F34" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>20261021_CMSUNIV_ODAG3_40_DAILY_2200_1</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>DAILY is due every day: the previous day</t>
         </is>
@@ -3392,11 +4616,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
@@ -3408,7 +4632,7 @@
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>One row per source. Three FDR (delegated entity) sources and two internal sources. Src_ID values and names are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>One row per source. Three FDR (delegated entity) sources, two internal sources that send files and two internal sources pulled from their tables with a query (SOURCE_LOAD). Src_ID values and names are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -3691,6 +4915,86 @@
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>UMAuth</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>AppealsDB</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -4013,7 +5317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4034,7 +5338,7 @@
     <row r="1" ht="64" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>One row per source and run type that gets batches. Assumed here: internal sources have DAILY, MNT and CMS; FDR sources have MNT and CMS (no daily files). Rpt_Dt_Sql_Txt gives the report dates of a scheduled batch; CMS rows need none because the dates come from the intake request. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>One row per source and run type that gets batches. Assumed here: internal sources (file and query) have DAILY, MNT and CMS; FDR sources have MNT and CMS (no daily files). Rpt_Dt_Sql_Txt gives the report dates of a scheduled batch; CMS rows need none because the dates come from the intake request. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -4531,12 +5835,12 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="E11" s="15" t="n">
@@ -4550,7 +5854,7 @@
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
+          <t>SELECT CAST({run_date} AS DATE) - 1 AS rpt_start, CAST({run_date} AS DATE) - 1 AS rpt_end</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
@@ -4590,12 +5894,12 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>CMS</t>
+          <t>MNT</t>
         </is>
       </c>
       <c r="E12" s="15" t="n">
@@ -4607,7 +5911,11 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H12" s="14" t="n"/>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
+        </is>
+      </c>
       <c r="I12" s="10" t="n">
         <v>1</v>
       </c>
@@ -4645,12 +5953,12 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>MNT</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="E13" s="15" t="n">
@@ -4662,11 +5970,7 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
+      <c r="H13" s="14" t="n"/>
       <c r="I13" s="10" t="n">
         <v>1</v>
       </c>
@@ -4704,12 +6008,12 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>CMS</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="E14" s="15" t="n">
@@ -4721,7 +6025,11 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H14" s="14" t="n"/>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>SELECT CAST({run_date} AS DATE) - 1 AS rpt_start, CAST({run_date} AS DATE) - 1 AS rpt_end</t>
+        </is>
+      </c>
       <c r="I14" s="10" t="n">
         <v>1</v>
       </c>
@@ -4759,7 +6067,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -4818,7 +6126,7 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -4855,6 +6163,348 @@
         </is>
       </c>
       <c r="M16" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M17" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="n"/>
+      <c r="I18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M18" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M22" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5594,6 +7244,347 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="112" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Optional: internal sources pulled by batch with their own SELECT (SOURCE_LOAD) instead of a file; such a source has no file config. Src_Conn_Cd is the Airflow Connection of the source's server; empty = the framework's own Teradata system (rows copied with one INSERT ... SELECT). Src_Sql_Txt is one SELECT in the source's dialect; {rpt_start}, {rpt_end}, {btch_id}, {run_ty}, ... are bound as parameters ($env is not replaced inside the query: name the real database). Its column names fill the staging columns of the same name. Table and column names here are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Src_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Src_Db_Ty</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Src_Conn_Cd</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Src_Sql_Txt</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Stg_Schema_Nm</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Stg_Table_Nm</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Core_Schema_Nm</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Core_Table_Nm</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(20) NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(32000) NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128) NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128) NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>TERADATA</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>SELECT a.Mbr_First_Nm AS MemberFirstName, a.Mbr_Last_Nm AS MemberLastName, a.Mbr_ID AS MemberID, a.Contract_ID AS ContractID, a.Auth_Nbr AS AuthorizationorClaimNumber, a.Rcvd_Dt AS Datetherequestwasreceived FROM CMSUNIV_SRC_DEV_V.UM_AUTH a WHERE a.Rcvd_Dt BETWEEN {rpt_start} AND {rpt_end}</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_FILELAND_$ENV_T</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_CORE_$ENV_T</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>SQLSERVER</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>cms_src_appeals_sqlsrv</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>SELECT m.FirstName AS MemberFirstName, m.LastName AS MemberLastName, m.MemberNumber AS MemberID, a.ContractId AS ContractID, a.AppealNumber AS AuthorizationorClaimNumber, CONVERT(varchar(10), a.ReceivedDate, 23) AS Datetherequestwasreceived FROM dbo.Appeal a JOIN dbo.Member m ON m.MemberKey = a.MemberKey WHERE a.ReceivedDate &gt;= {rpt_start} AND a.ReceivedDate &lt; DATEADD(day, 1, {rpt_end})</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_FILELAND_$ENV_T</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_CORE_$ENV_T</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6048,518 +8039,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="90" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="128" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Which content checks FILE_CHECK applies. CHARACTER_SET and COLUMN_VALUES apply to every table of the project: every line must be Latin text and every value must fit its target column (length, number, NOT NULL); all offending records go to the error file. The three ODAG3 '*' rows are the defaults for every ODAG3 source: header names, H / D / T record types and the trailer layout. The two rows with Include_Ind = 0 exclude the internal sources from the record type check, since their files have none (their trailer check does not apply either, because Src_File_Has_Trlr_Ind = 0). The header names here are the table's column names, as a placeholder: put the real header line of the ODAG3 file. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Project_Cd</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Table_Nm</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Src_ID</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Check_Cd</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Check_Val_Txt</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Include_Ind</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Active_Ind</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Created_Dtts</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Created_By</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_Dtts</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_By</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(63) DEFAULT '*' NOT NULL</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) DEFAULT '*' NOT NULL</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(8000)</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>HEADER_NAMES</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>MemberFirstName|MemberLastName|MemberID|ContractID|PlanBenefitPackage|FirstTierDownstreamandRelatedEntity|AuthorizationorClaimNumber|Datetherequestwasreceived|AORReceiptDate|WaiverofLiabilityReceiptDate|WasItaCleanClaim|WasTheRequestProcessedasanODorRecon|RequestDetermination|DateofDetermination|DateClaimReconsiderationwasPaid|DateWrittenNotificationprovidedToMember|DateWrittenNotificationProvidedtoProvider|DateForwardedtoIRE|Whomadetherequest|Issuedescriptionandtypeofservice|WasTheInitOrgDetReqtDeniedForLackOfMediNecessity|ExRMNumber|SourceUnique_ID|Filler2|Filler3</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>RECORD_TYPE</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>H,D,T</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>TRAILER</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>RECORD_TYPE,FILE_NAME,TOTAL_ROW_COUNT,TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>CHARACTER_SET</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>latin-1</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>COLUMN_VALUES</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>RECORD_TYPE</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>RECORD_TYPE</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Sample query sources select by batch ID
Both sample Src_Sql_Txt queries select the source rows by {btch_id}
instead of the report dates.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -7264,10 +7264,10 @@
     <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="112" customHeight="1">
+    <row r="1" ht="128" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Optional: internal sources pulled by batch with their own SELECT (SOURCE_LOAD) instead of a file; such a source has no file config. Src_Conn_Cd is the Airflow Connection of the source's server; empty = the framework's own Teradata system (rows copied with one INSERT ... SELECT). Src_Sql_Txt is one SELECT in the source's dialect; {rpt_start}, {rpt_end}, {btch_id}, {run_ty}, ... are bound as parameters ($env is not replaced inside the query: name the real database). Its column names fill the staging columns of the same name. Table and column names here are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Optional: internal sources pulled by batch with their own SELECT (SOURCE_LOAD) instead of a file; such a source has no file config. Src_Conn_Cd is the Airflow Connection of the source's server; empty = the framework's own Teradata system (rows copied with one INSERT ... SELECT). Src_Sql_Txt is one SELECT in the source's dialect, driven by the batch: here the source rows carry the framework's batch ID and {btch_id} selects them ({rpt_start}, {rpt_end}, {run_ty}, ... can be used too); every {name} is bound as a parameter ($env is not replaced inside the query: name the real database). Its column names fill the staging columns of the same name. Table and column names here are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -7449,7 +7449,7 @@
       <c r="E5" s="10" t="n"/>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>SELECT a.Mbr_First_Nm AS MemberFirstName, a.Mbr_Last_Nm AS MemberLastName, a.Mbr_ID AS MemberID, a.Contract_ID AS ContractID, a.Auth_Nbr AS AuthorizationorClaimNumber, a.Rcvd_Dt AS Datetherequestwasreceived FROM CMSUNIV_SRC_DEV_V.UM_AUTH a WHERE a.Rcvd_Dt BETWEEN {rpt_start} AND {rpt_end}</t>
+          <t>SELECT a.Mbr_First_Nm AS MemberFirstName, a.Mbr_Last_Nm AS MemberLastName, a.Mbr_ID AS MemberID, a.Contract_ID AS ContractID, a.Auth_Nbr AS AuthorizationorClaimNumber, a.Rcvd_Dt AS Datetherequestwasreceived FROM CMSUNIV_SRC_DEV_V.UM_AUTH a WHERE a.Btch_ID = {btch_id}</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>SELECT m.FirstName AS MemberFirstName, m.LastName AS MemberLastName, m.MemberNumber AS MemberID, a.ContractId AS ContractID, a.AppealNumber AS AuthorizationorClaimNumber, CONVERT(varchar(10), a.ReceivedDate, 23) AS Datetherequestwasreceived FROM dbo.Appeal a JOIN dbo.Member m ON m.MemberKey = a.MemberKey WHERE a.ReceivedDate &gt;= {rpt_start} AND a.ReceivedDate &lt; DATEADD(day, 1, {rpt_end})</t>
+          <t>SELECT m.FirstName AS MemberFirstName, m.LastName AS MemberLastName, m.MemberNumber AS MemberID, a.ContractId AS ContractID, a.AppealNumber AS AuthorizationorClaimNumber, CONVERT(varchar(10), a.ReceivedDate, 23) AS Datetherequestwasreceived FROM dbo.Appeal a JOIN dbo.Member m ON m.MemberKey = a.MemberKey WHERE a.Btch_ID = {btch_id}</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Schedule codes and batch calendar instead of SQL (Airflow / Teradata)
- ComplianceRunType: Sched_Cd (DAILY / WEEKLY / MONTHLY), Sched_Day_Cd
  (MON..SUN, 1..31, LAST), Sched_Week_Cd (n-th weekday 1..4 / LAST),
  Sched_Months_Txt (e.g. 1,4,7,10) and Sched_Window_Days (a missed run
  still creates the batch for the same report dates).
- ComplianceDataSetSourceXwalk.Rpt_Period_Cd: the built-in report periods
  (PREV_DAY, PREV_CALENDAR_WEEK, PREV_CALENDAR_MONTH, ...) counted from the
  scheduled date.
- Optional ComplianceBatchCalendar: batches on given request dates with
  given report dates, for every source of the run type (and table).
- Batch_Schedule_Sql_Txt / Rpt_Dt_Sql_Txt stay as the fallback when no code
  is set. validate-config checks the codes and the calendar rows.
- Sample metadata uses the codes; version 0.3.39.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -13,17 +13,18 @@
     <sheet name="ComplianceSourceSystem" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ComplianceRunType" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="ComplianceDataSetSourceXwalk" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ComplianceSourceFileConfig" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ComplianceSourceQueryConfig" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ComplianceTargetColumnConfig" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="ComplianceExportConfig" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ComplianceFileCheckConfig" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ComplianceRuleBinding" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ComplianceRequestInTake" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="ComplianceBatchOverride" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Airflow Variables" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Sample files" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Expected batches" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="ComplianceBatchCalendar" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ComplianceSourceFileConfig" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ComplianceSourceQueryConfig" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ComplianceTargetColumnConfig" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ComplianceExportConfig" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ComplianceFileCheckConfig" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ComplianceRuleBinding" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ComplianceRequestInTake" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="ComplianceBatchOverride" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Airflow Variables" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Sample files" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Expected batches" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -161,13 +162,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -584,14 +582,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Sources: three FDR sources (51 MedHOK, 130 OptumRx, 140 ESI) and two internal sources (10 Claims, 20 Appeals).</t>
+          <t>Sources: three FDR sources (51 MedHOK, 130 OptumRx, 140 ESI), two internal sources sending files (10 Claims, 20 Appeals) and two pulled with a query (30 UMAuth, 40 AppealsDB).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Run types: DAILY (scheduled, every day, for the previous day), MNT (scheduled, week of the 3rd Tuesday, for the previous month) and CMS (ad-hoc, requested through ComplianceRequestInTake, carry-forward allowed).</t>
+          <t>Run types: DAILY (scheduled, every day, for the previous day), MNT (scheduled, 3rd Monday, for the previous month) and CMS (ad-hoc, requested through ComplianceRequestInTake, carry-forward allowed).</t>
         </is>
       </c>
     </row>
@@ -732,6 +730,468 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="112" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Which columns of the staging and core tables the framework fills. Every other column of the staging table is a column of the file, in table order (the 25 ODAG3 columns here). The '*' rows apply to every CMSUNIV table; the row ID is one row per table. Btch_ID needs no row. When a file is loaded for a batch that already has rows in the core table, those rows are deleted by Btch_ID and the new rows are inserted. Value_Txt is only filled for two more codes these tables do not need: CONSTANT (a fixed value such as Y) and SQL (a SELECT returning one value, for example an audit ID from another table). Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Column_Nm</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Value_Cd</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Value_Txt</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) DEFAULT '*' NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(8000)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>StagingCreateDate</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>LOAD_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Universe_Vrsn</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>VERSION</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Run_Ty</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>RUN_TYPE</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>FileName</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>FILE_NAME</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Src_Data_Key</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>SOURCE_ID</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Load_Dtts</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>LOAD_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_Table3_2022_ID</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>ROW_SEQUENCE</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -941,7 +1401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1455,7 +1915,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1661,7 +2121,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1859,16 +2319,16 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="14" t="n">
         <v>46204</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="14" t="n">
         <v>46295</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H5" s="14" t="n">
         <v>46314</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="14" t="n">
         <v>46314</v>
       </c>
       <c r="J5" s="10" t="n"/>
@@ -1919,16 +2379,16 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="14" t="n">
         <v>46113</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="14" t="n">
         <v>46203</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="14" t="n">
         <v>46316</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="I6" s="14" t="n">
         <v>46316</v>
       </c>
       <c r="J6" s="10" t="n"/>
@@ -1961,7 +2421,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2168,7 +2628,7 @@
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="14" t="n">
         <v>46325</v>
       </c>
       <c r="H5" s="10" t="inlineStr">
@@ -2234,7 +2694,7 @@
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="14" t="n">
         <v>46326</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -2281,7 +2741,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2571,7 +3031,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2643,7 +3103,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_Claims_PYMT_C_22_CMS_20260701_20260930_20261019093000.txt</t>
         </is>
@@ -2675,7 +3135,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_OptumRx_PYMT_C_22_CMS_20260701_20260930_20261019093000.txt</t>
         </is>
@@ -2707,7 +3167,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_ESI_PYMT_C_22_CMS_20260701_20260930_20261019093000.txt</t>
         </is>
@@ -2739,7 +3199,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_Appeals_PYMT_C_22_CMS_20260701_20260930_20261019093000.txt</t>
         </is>
@@ -2771,7 +3231,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_MedHOK_PYMT_C_22_CMS_20260701_20260930_20261019093000.txt</t>
         </is>
@@ -2803,7 +3263,7 @@
           <t>DAILY</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_Claims_PYMT_C_22_DAILY_20261018_20261018_20261019093000.txt</t>
         </is>
@@ -2835,7 +3295,7 @@
           <t>DAILY</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_Appeals_PYMT_C_22_DAILY_20261018_20261018_20261019093000.txt</t>
         </is>
@@ -2867,7 +3327,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_Claims_PYMT_C_22_MNT_20260901_20260930_20261019093000.txt</t>
         </is>
@@ -2899,7 +3359,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_OptumRx_PYMT_C_22_MNT_20260901_20260930_20261019093000.txt</t>
         </is>
@@ -2931,7 +3391,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_ESI_PYMT_C_22_MNT_20260901_20260930_20261019093000.txt</t>
         </is>
@@ -2963,7 +3423,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_Appeals_PYMT_C_22_MNT_20260901_20260930_20261019093000.txt</t>
         </is>
@@ -2995,7 +3455,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_MedHOK_PYMT_C_22_MNT_20260901_20260930_20261019093000.txt</t>
         </is>
@@ -3027,7 +3487,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>CMSAuth_MedHOK_PYMT_C_17_MNT_20260901_20260930_20261019100000.txt</t>
         </is>
@@ -3043,7 +3503,7 @@
       <c r="A17" s="11" t="n"/>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="11" t="n"/>
-      <c r="D17" s="16" t="n"/>
+      <c r="D17" s="15" t="n"/>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
     </row>
@@ -3055,7 +3515,7 @@
       </c>
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">H|MemberFirstName|MemberLastName|MemberID|ContractID|PlanBenefitPackage|FirstTierDownstreamandRelatedEntity|AuthorizationorClaimNumber|Datetherequestwasreceived|AORReceiptDate|WaiverofLiabilityReceiptDate|WasItaCleanClaim|WasTheRequestProcessedasanODorRecon|RequestDetermination|DateofDetermination|DateClaimReconsiderationwasPaid|DateWrittenNotificationprovidedToMember|DateWrittenNotificationProvidedtoProvider|DateForwardedtoIRE|Whomadetherequest|Issuedescriptionandtypeofservice|WasTheInitOrgDetReqtDeniedForLackOfMediNecessity|ExRMNumber|SourceUnique_ID|Filler2|Filler3
 D|First1|Last1|M0001|H1234|001||||||||||||||||||SRC51-1||
@@ -3079,7 +3539,7 @@
       </c>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">MemberFirstName|MemberLastName|MemberID|ContractID|PlanBenefitPackage|FirstTierDownstreamandRelatedEntity|AuthorizationorClaimNumber|Datetherequestwasreceived|AORReceiptDate|WaiverofLiabilityReceiptDate|WasItaCleanClaim|WasTheRequestProcessedasanODorRecon|RequestDetermination|DateofDetermination|DateClaimReconsiderationwasPaid|DateWrittenNotificationprovidedToMember|DateWrittenNotificationProvidedtoProvider|DateForwardedtoIRE|Whomadetherequest|Issuedescriptionandtypeofservice|WasTheInitOrgDetReqtDeniedForLackOfMediNecessity|ExRMNumber|SourceUnique_ID|Filler2|Filler3
 First1|Last1|M0001|H1234|001||||||||||||||||||SRC10-1||
@@ -3102,7 +3562,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3171,7 +3631,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="16" t="n">
         <v>46311</v>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -3189,10 +3649,10 @@
           <t>Claims</t>
         </is>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="16" t="n">
         <v>46310</v>
       </c>
-      <c r="F4" s="17" t="n">
+      <c r="F4" s="16" t="n">
         <v>46310</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
@@ -3207,7 +3667,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="16" t="n">
         <v>46311</v>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -3225,10 +3685,10 @@
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="16" t="n">
         <v>46310</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="16" t="n">
         <v>46310</v>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -3243,7 +3703,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="16" t="n">
         <v>46311</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -3261,10 +3721,10 @@
           <t>UMAuth</t>
         </is>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="16" t="n">
         <v>46310</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="16" t="n">
         <v>46310</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -3279,7 +3739,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="16" t="n">
         <v>46311</v>
       </c>
       <c r="B7" s="11" t="inlineStr">
@@ -3297,10 +3757,10 @@
           <t>AppealsDB</t>
         </is>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="16" t="n">
         <v>46310</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="16" t="n">
         <v>46310</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
@@ -3315,7 +3775,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -3333,10 +3793,10 @@
           <t>Claims</t>
         </is>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
@@ -3351,7 +3811,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -3369,10 +3829,10 @@
           <t>OptumRx</t>
         </is>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -3387,7 +3847,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -3405,10 +3865,10 @@
           <t>ESI</t>
         </is>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
@@ -3423,7 +3883,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -3441,10 +3901,10 @@
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="F11" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -3459,7 +3919,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -3477,10 +3937,10 @@
           <t>UMAuth</t>
         </is>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -3495,7 +3955,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -3513,10 +3973,10 @@
           <t>AppealsDB</t>
         </is>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -3531,7 +3991,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -3549,10 +4009,10 @@
           <t>MedHOK</t>
         </is>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="16" t="n">
         <v>46204</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -3567,7 +4027,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -3585,10 +4045,10 @@
           <t>Claims</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="16" t="n">
         <v>46313</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="16" t="n">
         <v>46313</v>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -3603,7 +4063,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="n">
+      <c r="A16" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -3621,10 +4081,10 @@
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="16" t="n">
         <v>46313</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="16" t="n">
         <v>46313</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -3639,7 +4099,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="n">
+      <c r="A17" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -3657,10 +4117,10 @@
           <t>UMAuth</t>
         </is>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="16" t="n">
         <v>46313</v>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="16" t="n">
         <v>46313</v>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -3675,7 +4135,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="n">
+      <c r="A18" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -3693,10 +4153,10 @@
           <t>AppealsDB</t>
         </is>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="16" t="n">
         <v>46313</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="16" t="n">
         <v>46313</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -3711,7 +4171,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="n">
+      <c r="A19" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -3729,10 +4189,10 @@
           <t>Claims</t>
         </is>
       </c>
-      <c r="E19" s="17" t="n">
+      <c r="E19" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F19" s="17" t="n">
+      <c r="F19" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -3742,12 +4202,12 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -3765,10 +4225,10 @@
           <t>OptumRx</t>
         </is>
       </c>
-      <c r="E20" s="17" t="n">
+      <c r="E20" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F20" s="17" t="n">
+      <c r="F20" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -3778,12 +4238,12 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="n">
+      <c r="A21" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B21" s="11" t="inlineStr">
@@ -3801,10 +4261,10 @@
           <t>ESI</t>
         </is>
       </c>
-      <c r="E21" s="17" t="n">
+      <c r="E21" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F21" s="17" t="n">
+      <c r="F21" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -3814,12 +4274,12 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="n">
+      <c r="A22" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -3837,10 +4297,10 @@
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n">
+      <c r="E22" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F22" s="17" t="n">
+      <c r="F22" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -3850,12 +4310,12 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="n">
+      <c r="A23" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -3873,10 +4333,10 @@
           <t>UMAuth</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n">
+      <c r="E23" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F23" s="17" t="n">
+      <c r="F23" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -3886,12 +4346,12 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -3909,10 +4369,10 @@
           <t>AppealsDB</t>
         </is>
       </c>
-      <c r="E24" s="17" t="n">
+      <c r="E24" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F24" s="17" t="n">
+      <c r="F24" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -3922,12 +4382,12 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
+      <c r="A25" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -3945,10 +4405,10 @@
           <t>MedHOK</t>
         </is>
       </c>
-      <c r="E25" s="17" t="n">
+      <c r="E25" s="16" t="n">
         <v>46266</v>
       </c>
-      <c r="F25" s="17" t="n">
+      <c r="F25" s="16" t="n">
         <v>46295</v>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -3958,12 +4418,12 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>MNT window (Sun 18 - Thu 22 Oct, 3rd Tuesday = 20 Oct): September</t>
+          <t>MNT on the 3rd Monday (19 Oct) and 5 days after: September</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="n">
+      <c r="A26" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -3981,10 +4441,10 @@
           <t>Claims</t>
         </is>
       </c>
-      <c r="E26" s="17" t="n">
+      <c r="E26" s="16" t="n">
         <v>46314</v>
       </c>
-      <c r="F26" s="17" t="n">
+      <c r="F26" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
@@ -3999,7 +4459,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n">
+      <c r="A27" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -4017,10 +4477,10 @@
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E27" s="17" t="n">
+      <c r="E27" s="16" t="n">
         <v>46314</v>
       </c>
-      <c r="F27" s="17" t="n">
+      <c r="F27" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -4035,7 +4495,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n">
+      <c r="A28" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -4053,10 +4513,10 @@
           <t>UMAuth</t>
         </is>
       </c>
-      <c r="E28" s="17" t="n">
+      <c r="E28" s="16" t="n">
         <v>46314</v>
       </c>
-      <c r="F28" s="17" t="n">
+      <c r="F28" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -4071,7 +4531,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n">
+      <c r="A29" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="B29" s="11" t="inlineStr">
@@ -4089,10 +4549,10 @@
           <t>AppealsDB</t>
         </is>
       </c>
-      <c r="E29" s="17" t="n">
+      <c r="E29" s="16" t="n">
         <v>46314</v>
       </c>
-      <c r="F29" s="17" t="n">
+      <c r="F29" s="16" t="n">
         <v>46314</v>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -4107,7 +4567,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="n">
+      <c r="A30" s="16" t="n">
         <v>46316</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -4125,10 +4585,10 @@
           <t>ESI</t>
         </is>
       </c>
-      <c r="E30" s="17" t="n">
+      <c r="E30" s="16" t="n">
         <v>46113</v>
       </c>
-      <c r="F30" s="17" t="n">
+      <c r="F30" s="16" t="n">
         <v>46203</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -4143,7 +4603,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="n">
+      <c r="A31" s="16" t="n">
         <v>46316</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
@@ -4161,10 +4621,10 @@
           <t>Claims</t>
         </is>
       </c>
-      <c r="E31" s="17" t="n">
+      <c r="E31" s="16" t="n">
         <v>46315</v>
       </c>
-      <c r="F31" s="17" t="n">
+      <c r="F31" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="G31" s="11" t="inlineStr">
@@ -4179,7 +4639,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="n">
+      <c r="A32" s="16" t="n">
         <v>46316</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -4197,10 +4657,10 @@
           <t>Appeals</t>
         </is>
       </c>
-      <c r="E32" s="17" t="n">
+      <c r="E32" s="16" t="n">
         <v>46315</v>
       </c>
-      <c r="F32" s="17" t="n">
+      <c r="F32" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -4215,7 +4675,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="n">
+      <c r="A33" s="16" t="n">
         <v>46316</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
@@ -4233,10 +4693,10 @@
           <t>UMAuth</t>
         </is>
       </c>
-      <c r="E33" s="17" t="n">
+      <c r="E33" s="16" t="n">
         <v>46315</v>
       </c>
-      <c r="F33" s="17" t="n">
+      <c r="F33" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -4251,7 +4711,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="n">
+      <c r="A34" s="16" t="n">
         <v>46316</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -4269,10 +4729,10 @@
           <t>AppealsDB</t>
         </is>
       </c>
-      <c r="E34" s="17" t="n">
+      <c r="E34" s="16" t="n">
         <v>46315</v>
       </c>
-      <c r="F34" s="17" t="n">
+      <c r="F34" s="16" t="n">
         <v>46315</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
@@ -5014,7 +5474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5023,17 +5483,22 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="100" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="64" customHeight="1">
+    <row r="1" ht="112" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Batch_Schedule_Sql_Txt says WHEN scheduled batches are created (one row = due that day). CMS is ad-hoc: no schedule, and Carry_Fwd_Ind = 1 allows an approved REUSE override to carry an earlier batch's data forward. SLA_Days are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>Sched_Cd / Sched_Day_Cd / Sched_Week_Cd / Sched_Months_Txt say WHEN scheduled batches are created: DAILY; WEEKLY on a day (MON ... SUN); MONTHLY on a day number (1 ... 31, LAST) or the n-th weekday (Sched_Day_Cd MON ... SUN with Sched_Week_Cd 1 ... 4 or LAST), optionally only in some months (Sched_Months_Txt '1,4,7,10'). Sched_Window_Days lets a missed run still create the batch that many days (same report dates). Batch_Schedule_Sql_Txt is a fallback for a schedule the codes cannot express. CMS is ad-hoc: no schedule, and Carry_Fwd_Ind = 1 allows an approved REUSE override to carry an earlier batch's data forward. SLA_Days are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -5070,25 +5535,50 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
+          <t>Sched_Cd</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Sched_Day_Cd</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Sched_Week_Cd</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Sched_Months_Txt</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Sched_Window_Days</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
           <t>Active_Ind</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>Created_Dtts</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Created_By</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>Updated_Dtts</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Updated_By</t>
         </is>
@@ -5127,25 +5617,50 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(5)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(5)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(40)</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
           <t>SMALLINT DEFAULT 1 NOT NULL</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="P4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
@@ -5173,30 +5688,37 @@
       <c r="E5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>SELECT 1 AS due</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="n">
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="L5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="P5" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5210,7 +5732,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Monthly submission, created in the week of the 3rd Tuesday</t>
+          <t>Monthly submission, created on the 3rd Monday (5 days to catch up a missed run)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -5224,33 +5746,45 @@
       <c r="E6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>SELECT tue AS period_dt
-FROM (SELECT CAST({run_date} AS DATE) + (3 - TD_DAY_OF_WEEK(CAST({run_date} AS DATE))) AS tue) x
-WHERE TD_DAY_OF_WEEK(CAST({run_date} AS DATE)) &lt;= 5
-  AND (EXTRACT(DAY FROM tue) - 1) / 7 + 1 = 3</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="n">
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>MONTHLY</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>MON</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="P6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5278,26 +5812,33 @@
       <c r="E7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="10" t="n">
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="L7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="O7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="P7" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5305,7 +5846,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5317,7 +5858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5328,17 +5869,18 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="110" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="64" customHeight="1">
+    <row r="1" ht="112" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>One row per source and run type that gets batches. Assumed here: internal sources (file and query) have DAILY, MNT and CMS; FDR sources have MNT and CMS (no daily files). Rpt_Dt_Sql_Txt gives the report dates of a scheduled batch; CMS rows need none because the dates come from the intake request. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>One row per source and run type that gets batches. Assumed here: internal sources (file and query) have DAILY, MNT and CMS; FDR sources have MNT and CMS (no daily files). Rpt_Period_Cd gives the report dates of a scheduled batch, counted from its scheduled date: PREV_DAY, PREV_CALENDAR_WEEK, PREV_CALENDAR_MONTH, PREV_CALENDAR_QUARTER, PREV_CALENDAR_YEAR, CURRENT_CALENDAR_MONTH, ROLLING_1_MONTH, PREV_N_DAYS(n), PREV_WEEK_SAME_DAY(n), SAME_DAY, ANNUAL_WINDOW(MM-DD,MM-DD); Rpt_Dt_Sql_Txt is a fallback for anything else. CMS rows need none because the dates come from the intake request. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -5385,25 +5927,30 @@
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
+          <t>Rpt_Period_Cd</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
           <t>Active_Ind</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>Created_Dtts</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>Created_By</t>
         </is>
       </c>
-      <c r="L3" s="8" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>Updated_Dtts</t>
         </is>
       </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Updated_By</t>
         </is>
@@ -5452,25 +5999,30 @@
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
           <t>SMALLINT DEFAULT 1 NOT NULL</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
@@ -5497,7 +6049,7 @@
           <t>DAILY</t>
         </is>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F5" s="10" t="n"/>
@@ -5506,30 +6058,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>SELECT CAST({run_date} AS DATE) - 1 AS rpt_start, CAST({run_date} AS DATE) - 1 AS rpt_end</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="n">
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>PREV_DAY</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5556,7 +6109,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F6" s="10" t="n"/>
@@ -5565,30 +6118,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="n">
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5615,7 +6169,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F7" s="10" t="n"/>
@@ -5624,26 +6178,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H7" s="14" t="n"/>
-      <c r="I7" s="10" t="n">
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5670,7 +6225,7 @@
           <t>DAILY</t>
         </is>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F8" s="10" t="n"/>
@@ -5679,30 +6234,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
-        <is>
-          <t>SELECT CAST({run_date} AS DATE) - 1 AS rpt_start, CAST({run_date} AS DATE) - 1 AS rpt_end</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="n">
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>PREV_DAY</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N8" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5729,7 +6285,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F9" s="10" t="n"/>
@@ -5738,30 +6294,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="n">
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5788,7 +6345,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F10" s="10" t="n"/>
@@ -5797,26 +6354,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H10" s="14" t="n"/>
-      <c r="I10" s="10" t="n">
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="10" t="n"/>
+      <c r="J10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N10" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5843,7 +6401,7 @@
           <t>DAILY</t>
         </is>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F11" s="10" t="n"/>
@@ -5852,30 +6410,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>SELECT CAST({run_date} AS DATE) - 1 AS rpt_start, CAST({run_date} AS DATE) - 1 AS rpt_end</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="n">
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>PREV_DAY</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5902,7 +6461,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F12" s="10" t="n"/>
@@ -5911,30 +6470,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I12" s="10" t="n">
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M12" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N12" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -5961,7 +6521,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F13" s="10" t="n"/>
@@ -5970,26 +6530,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H13" s="14" t="n"/>
-      <c r="I13" s="10" t="n">
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="10" t="n"/>
+      <c r="J13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M13" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6016,7 +6577,7 @@
           <t>DAILY</t>
         </is>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F14" s="10" t="n"/>
@@ -6025,30 +6586,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
-        <is>
-          <t>SELECT CAST({run_date} AS DATE) - 1 AS rpt_start, CAST({run_date} AS DATE) - 1 AS rpt_end</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="n">
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>PREV_DAY</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M14" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N14" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6075,7 +6637,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F15" s="10" t="n"/>
@@ -6084,30 +6646,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="n">
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M15" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N15" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6134,7 +6697,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F16" s="10" t="n"/>
@@ -6143,26 +6706,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H16" s="14" t="n"/>
-      <c r="I16" s="10" t="n">
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="10" t="n"/>
+      <c r="J16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M16" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N16" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6189,7 +6753,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F17" s="10" t="n"/>
@@ -6198,30 +6762,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="n">
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M17" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N17" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6248,7 +6813,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F18" s="10" t="n"/>
@@ -6257,26 +6822,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H18" s="14" t="n"/>
-      <c r="I18" s="10" t="n">
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="10" t="n"/>
+      <c r="J18" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M18" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N18" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6303,7 +6869,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F19" s="10" t="n"/>
@@ -6312,30 +6878,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="n">
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L19" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6362,7 +6929,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="E20" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F20" s="10" t="n"/>
@@ -6371,26 +6938,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="10" t="n">
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N20" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6417,7 +6985,7 @@
           <t>MNT</t>
         </is>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F21" s="10" t="n"/>
@@ -6426,30 +6994,31 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>SELECT ADD_MONTHS(p - EXTRACT(DAY FROM p) + 1, -1) AS rpt_start, p - EXTRACT(DAY FROM p) AS rpt_end FROM (SELECT CAST({period_dt} AS DATE) AS p) d</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="n">
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>PREV_CALENDAR_MONTH</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N21" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6476,7 +7045,7 @@
           <t>CMS</t>
         </is>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="E22" s="14" t="n">
         <v>46023</v>
       </c>
       <c r="F22" s="10" t="n"/>
@@ -6485,26 +7054,27 @@
           <t>2200</t>
         </is>
       </c>
-      <c r="H22" s="14" t="n"/>
-      <c r="I22" s="10" t="n">
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="10" t="n"/>
+      <c r="J22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J22" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>(default USER)</t>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
         </is>
       </c>
       <c r="L22" s="11" t="inlineStr">
         <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
+          <t>(default USER)</t>
         </is>
       </c>
       <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="N22" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6512,13 +7082,213 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="80" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Optional: batches on given dates with given report dates, for what the schedule codes do not cover (an extra or moved submission). On Req_Dt_Key BATCH_CREATION creates a batch for these report dates for every source of the run type in the crosswalk (Table_Nm '*' = every table). Here: an extra MNT batch for August, created on 2026-11-03. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Run_Ty</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Req_Dt_Key</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Rpt_Start_Dt_Key</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Rpt_End_Dt_Key</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) DEFAULT '*' NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(20) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>DATE NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>DATE NOT NULL</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>DATE NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>MNT</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>46329</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>46235</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>46265</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6781,7 +7551,7 @@
           <t>51</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>CMSAuth_MedHOK_PYMT_C_{VERSION}_{RUNTY}_{RPTSTART}_{RPTEND}_{TS}.txt</t>
         </is>
@@ -6875,7 +7645,7 @@
           <t>130</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>CMSAuth_OptumRx_PYMT_C_{VERSION}_{RUNTY}_{RPTSTART}_{RPTEND}_{TS}.txt</t>
         </is>
@@ -6969,7 +7739,7 @@
           <t>140</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>CMSAuth_ESI_PYMT_C_{VERSION}_{RUNTY}_{RPTSTART}_{RPTEND}_{TS}.txt</t>
         </is>
@@ -7063,7 +7833,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>CMSAuth_Claims_PYMT_C_{VERSION}_{RUNTY}_{RPTSTART}_{RPTEND}_{TS}.txt</t>
         </is>
@@ -7157,7 +7927,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>CMSAuth_Appeals_PYMT_C_{VERSION}_{RUNTY}_{RPTSTART}_{RPTEND}_{TS}.txt</t>
         </is>
@@ -7238,7 +8008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7577,466 +8347,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="112" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Which columns of the staging and core tables the framework fills. Every other column of the staging table is a column of the file, in table order (the 25 ODAG3 columns here). The '*' rows apply to every CMSUNIV table; the row ID is one row per table. Btch_ID needs no row. When a file is loaded for a batch that already has rows in the core table, those rows are deleted by Btch_ID and the new rows are inserted. Value_Txt is only filled for two more codes these tables do not need: CONSTANT (a fixed value such as Y) and SQL (a SELECT returning one value, for example an audit ID from another table). Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Project_Cd</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Table_Nm</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Column_Nm</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Value_Cd</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Value_Txt</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Active_Ind</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Created_Dtts</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Created_By</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_Dtts</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_By</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(63) DEFAULT '*' NOT NULL</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(128) NOT NULL</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(8000)</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>StagingCreateDate</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>LOAD_TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Universe_Vrsn</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>VERSION</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Run_Ty</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>RUN_TYPE</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>FileName</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>FILE_NAME</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Src_Data_Key</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>SOURCE_ID</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Load_Dtts</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>LOAD_TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>ODAG_DE_Table3_2022_ID</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>ROW_SEQUENCE</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Crosswalk run type lists, per-project report periods, RANGE period code; rename to ComplianceInternalSourceConfig (0.3.43)
- ComplianceDataSetSourceXwalk.Run_Ty lists run types (one row per table and source); a row for one
  run type replaces the list's entry while effective, Include_Ind = 0 switches it off
- ComplianceRunTypePeriod: report period per project / table and run type
- RANGE(DAY|WEEK|MONTH|QUARTER|YEAR, back, length) period code
- ComplianceSourceQueryConfig renamed to ComplianceInternalSourceConfig
- validate-config, deployment guide, runbook and sample metadata updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
+++ b/airflow/compliance_framework/examples/cmsuniv_odag3_sample_metadata.xlsx
@@ -12,19 +12,20 @@
     <sheet name="ComplianceTable" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ComplianceSourceSystem" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ComplianceRunType" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ComplianceDataSetSourceXwalk" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ComplianceBatchCalendar" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ComplianceSourceFileConfig" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ComplianceSourceQueryConfig" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="ComplianceTargetColumnConfig" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ComplianceExportConfig" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ComplianceFileCheckConfig" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ComplianceRuleBinding" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="ComplianceRequestInTake" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="ComplianceBatchOverride" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Airflow Variables" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Sample files" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Expected batches" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="ComplianceRunTypePeriod" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ComplianceDataSetSourceXwalk" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ComplianceBatchCalendar" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ComplianceSourceFileConfig" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ComplianceInternalSourceConfig" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ComplianceTargetColumnConfig" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ComplianceExportConfig" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ComplianceFileCheckConfig" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ComplianceRuleBinding" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="ComplianceRequestInTake" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="ComplianceBatchOverride" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Airflow Variables" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Sample files" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Expected batches" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -620,7 +621,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>One tab per metadata table that needs rows, in the order to load them: ComplianceProject, ComplianceSourceSystem, ComplianceTable (optional), ComplianceRunType, ComplianceDataSetSourceXwalk, ComplianceBatchCalendar (optional), ComplianceSourceFileConfig, ComplianceSourceQueryConfig (optional), ComplianceTargetColumnConfig, ComplianceExportConfig (optional), ComplianceFileCheckConfig, ComplianceRuleBinding (optional), ComplianceRequestInTake (one row per CMS request), ComplianceBatchOverride (only for a carry-forward or a reopen).</t>
+          <t>One tab per metadata table that needs rows, in the order to load them: ComplianceProject, ComplianceSourceSystem, ComplianceTable (optional), ComplianceRunType, ComplianceRunTypePeriod, ComplianceDataSetSourceXwalk, ComplianceBatchCalendar (optional), ComplianceSourceFileConfig, ComplianceInternalSourceConfig (optional), ComplianceTargetColumnConfig, ComplianceExportConfig (optional), ComplianceFileCheckConfig, ComplianceRuleBinding (optional), ComplianceRequestInTake (one row per CMS request), ComplianceBatchOverride (only for a carry-forward or a reopen).</t>
         </is>
       </c>
     </row>
@@ -730,6 +731,347 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="128" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Optional: internal sources pulled by batch with their own SELECT (SOURCE_LOAD) instead of a file; such a source has no file config. Src_Conn_Cd is the Airflow Connection of the source's server; empty = the framework's own Teradata system (rows copied with one INSERT ... SELECT). Src_Sql_Txt is one SELECT in the source's dialect, driven by the batch: here the source rows carry the framework's batch ID and {btch_id} selects them ({rpt_start}, {rpt_end}, {run_ty}, ... can be used too); every {name} is bound as a parameter ($env is not replaced inside the query: name the real database). Its column names fill the staging columns of the same name. Table and column names here are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Src_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Src_Db_Ty</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Src_Conn_Cd</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Src_Sql_Txt</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Stg_Schema_Nm</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Stg_Table_Nm</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Core_Schema_Nm</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Core_Table_Nm</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(20) NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(32000) NOT NULL</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128) NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(128) NOT NULL</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>TERADATA</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>SELECT a.Mbr_First_Nm AS MemberFirstName, a.Mbr_Last_Nm AS MemberLastName, a.Mbr_ID AS MemberID, a.Contract_ID AS ContractID, a.Auth_Nbr AS AuthorizationorClaimNumber, a.Rcvd_Dt AS Datetherequestwasreceived FROM CMSUNIV_SRC_DEV_V.UM_AUTH a WHERE a.Btch_ID = {btch_id}</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_FILELAND_$ENV_T</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_CORE_$ENV_T</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>SQLSERVER</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>cms_src_appeals_sqlsrv</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>SELECT m.FirstName AS MemberFirstName, m.LastName AS MemberLastName, m.MemberNumber AS MemberID, a.ContractId AS ContractID, a.AppealNumber AS AuthorizationorClaimNumber, CONVERT(varchar(10), a.ReceivedDate, 23) AS Datetherequestwasreceived FROM dbo.Appeal a JOIN dbo.Member m ON m.MemberKey = a.MemberKey WHERE a.Btch_ID = {btch_id}</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_FILELAND_$ENV_T</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV_CORE_$ENV_T</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG_DE_TABLE3_2022</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1191,7 +1533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1401,7 +1743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2019,7 +2361,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2225,7 +2567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2525,7 +2867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2845,7 +3187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3135,7 +3477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3666,7 +4008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5962,29 +6304,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="110" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="32" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="112" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>One row per source and run type that gets batches. Assumed here: internal sources (file and query) have DAILY, MNT and CMS; FDR sources have MNT and CMS (no daily files). Rpt_Period_Cd gives the report dates of a scheduled batch, counted from its scheduled date: PREV_DAY, PREV_CALENDAR_WEEK, PREV_CALENDAR_MONTH, PREV_CALENDAR_QUARTER, PREV_CALENDAR_YEAR, CURRENT_CALENDAR_MONTH, ROLLING_1_MONTH, PREV_N_DAYS(n), PREV_WEEK_SAME_DAY(n), SAME_DAY, ANNUAL_WINDOW(MM-DD,MM-DD); Rpt_Dt_Sql_Txt is a fallback for anything else. CMS rows need none because the dates come from the intake request. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+          <t>The report dates of a scheduled run type for the project, counted from the batch's scheduled date. Table_Nm '*' = every table; a row for one table wins over '*', and Rpt_Period_Cd on a crosswalk row wins over both. Codes: PREV_DAY, PREV_CALENDAR_WEEK, PREV_CALENDAR_MONTH, PREV_CALENDAR_QUARTER, PREV_CALENDAR_YEAR, CURRENT_CALENDAR_MONTH, ROLLING_1_MONTH, PREV_N_DAYS(n), PREV_WEEK_SAME_DAY(n), SAME_DAY, ANNUAL_WINDOW(MM-DD,MM-DD), and RANGE(DAY|WEEK|MONTH|QUARTER|YEAR, back, length) for any other range, e.g. RANGE(WEEK,5,1) = the Monday-Sunday week 5 weeks back. Ad-hoc run types (CMS) need none: the dates come from the intake request. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
         </is>
       </c>
     </row>
@@ -6001,60 +6338,35 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Src_ID</t>
+          <t>Run_Ty</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Run_Ty</t>
+          <t>Rpt_Period_Cd</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Effective_Start_Dt_Key</t>
+          <t>Active_Ind</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Effective_End_Dt_Key</t>
+          <t>Created_Dtts</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Cmplnc_Vrsn</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Rpt_Dt_Sql_Txt</t>
+          <t>Updated_Dtts</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Rpt_Period_Cd</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>Active_Ind</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>Created_Dtts</t>
-        </is>
-      </c>
-      <c r="L3" s="8" t="inlineStr">
-        <is>
-          <t>Created_By</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_Dtts</t>
-        </is>
-      </c>
-      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Updated_By</t>
         </is>
@@ -6068,65 +6380,40 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(63) NOT NULL</t>
+          <t>VARCHAR(63) DEFAULT '*' NOT NULL</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(30) NOT NULL</t>
+          <t>VARCHAR(20) NOT NULL</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20) NOT NULL</t>
+          <t>VARCHAR(60) NOT NULL</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>DATE NOT NULL</t>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10) NOT NULL</t>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(8000)</t>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(60)</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="L4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
         </is>
@@ -6140,53 +6427,38 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>ODAG3</t>
+          <t>*</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
           <t>DAILY</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>PREV_DAY</t>
         </is>
       </c>
-      <c r="J5" s="10" t="n">
+      <c r="E5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N5" s="11" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -6200,985 +6472,38 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>ODAG3</t>
+          <t>*</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
           <t>MNT</t>
         </is>
       </c>
-      <c r="E6" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="n"/>
-      <c r="I6" s="13" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>PREV_CALENDAR_MONTH</t>
         </is>
       </c>
-      <c r="J6" s="10" t="n">
+      <c r="E6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="n"/>
-      <c r="I7" s="10" t="n"/>
-      <c r="J7" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M7" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N7" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>DAILY</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="n"/>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>PREV_DAY</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L8" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M8" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N8" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>MNT</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="n"/>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>PREV_CALENDAR_MONTH</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M9" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N9" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="n"/>
-      <c r="I10" s="10" t="n"/>
-      <c r="J10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L10" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M10" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N10" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>DAILY</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="n"/>
-      <c r="I11" s="13" t="inlineStr">
-        <is>
-          <t>PREV_DAY</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M11" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N11" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>MNT</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="n"/>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>PREV_CALENDAR_MONTH</t>
-        </is>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M12" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N12" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="n"/>
-      <c r="I13" s="10" t="n"/>
-      <c r="J13" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L13" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M13" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N13" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>DAILY</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="n"/>
-      <c r="I14" s="13" t="inlineStr">
-        <is>
-          <t>PREV_DAY</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L14" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M14" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N14" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>MNT</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="n"/>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>PREV_CALENDAR_MONTH</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L15" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M15" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N15" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="10" t="n"/>
-      <c r="J16" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L16" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M16" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N16" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>MNT</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="n"/>
-      <c r="I17" s="13" t="inlineStr">
-        <is>
-          <t>PREV_CALENDAR_MONTH</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L17" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M17" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N17" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="n"/>
-      <c r="I18" s="10" t="n"/>
-      <c r="J18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L18" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M18" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N18" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>MNT</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="n"/>
-      <c r="I19" s="13" t="inlineStr">
-        <is>
-          <t>PREV_CALENDAR_MONTH</t>
-        </is>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L19" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N19" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H20" s="12" t="n"/>
-      <c r="I20" s="10" t="n"/>
-      <c r="J20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L20" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M20" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N20" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>140</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>MNT</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="n"/>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>PREV_CALENDAR_MONTH</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L21" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M21" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N21" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>140</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>46023</v>
-      </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="H22" s="12" t="n"/>
-      <c r="I22" s="10" t="n"/>
-      <c r="J22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="L22" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="M22" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="N22" s="11" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>(default USER)</t>
         </is>
@@ -7186,13 +6511,621 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="110" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="96" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>One row per table and source, Run_Ty lists its run types. Assumed here: internal sources (file and query) have DAILY, MNT and CMS; FDR sources have MNT and CMS (no daily files). The report dates come from ComplianceRunTypePeriod. A row for one run type replaces the list's entry for that run type while it is effective (its own version, dates or Rpt_Period_Cd), and Include_Ind = 0 on it switches that run type off for the source. Rpt_Dt_Sql_Txt is a fallback for dates no code expresses. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Src_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Run_Ty</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Effective_Start_Dt_Key</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Effective_End_Dt_Key</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Cmplnc_Vrsn</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Rpt_Dt_Sql_Txt</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Rpt_Period_Cd</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Include_Ind</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Active_Ind</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Created_Dtts</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_Dtts</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Updated_By</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(63) NOT NULL</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30) NOT NULL</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(200) NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>DATE NOT NULL</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(10) NOT NULL</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(8000)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>SMALLINT DEFAULT 1 NOT NULL</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>DAILY,MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>DAILY,MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>DAILY,MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N7" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O7" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>DAILY,MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="10" t="n"/>
+      <c r="J9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O9" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="10" t="n"/>
+      <c r="J10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N10" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O10" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CMSUNIV</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>ODAG3</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>MNT,CMS</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="10" t="n"/>
+      <c r="J11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
+        <is>
+          <t>(default CURRENT_TIMESTAMP(6))</t>
+        </is>
+      </c>
+      <c r="O11" s="11" t="inlineStr">
+        <is>
+          <t>(default USER)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7392,7 +7325,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8110,345 +8043,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="128" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Optional: internal sources pulled by batch with their own SELECT (SOURCE_LOAD) instead of a file; such a source has no file config. Src_Conn_Cd is the Airflow Connection of the source's server; empty = the framework's own Teradata system (rows copied with one INSERT ... SELECT). Src_Sql_Txt is one SELECT in the source's dialect, driven by the batch: here the source rows carry the framework's batch ID and {btch_id} selects them ({rpt_start}, {rpt_end}, {run_ty}, ... can be used too); every {name} is bound as a parameter ($env is not replaced inside the query: name the real database). Its column names fill the staging columns of the same name. Table and column names here are examples. Columns are exactly those of the table, in the order of the DDL; the second row is each column's definition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Project_Cd</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Table_Nm</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Src_ID</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Src_Db_Ty</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Src_Conn_Cd</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Src_Sql_Txt</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Stg_Schema_Nm</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Stg_Table_Nm</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Core_Schema_Nm</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>Core_Table_Nm</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>Active_Ind</t>
-        </is>
-      </c>
-      <c r="L3" s="8" t="inlineStr">
-        <is>
-          <t>Created_Dtts</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>Created_By</t>
-        </is>
-      </c>
-      <c r="N3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_Dtts</t>
-        </is>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>Updated_By</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(63) NOT NULL</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(30) NOT NULL</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(20) NOT NULL</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(32000) NOT NULL</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(128) NOT NULL</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(63) NOT NULL</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(128) NOT NULL</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(63) NOT NULL</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>SMALLINT DEFAULT 1 NOT NULL</t>
-        </is>
-      </c>
-      <c r="L4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-      <c r="N4" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP(6) WITH TIME ZONE DEFAULT CURRENT_TIMESTAMP(6) NOT NULL</t>
-        </is>
-      </c>
-      <c r="O4" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100) DEFAULT USER NOT NULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>TERADATA</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>SELECT a.Mbr_First_Nm AS MemberFirstName, a.Mbr_Last_Nm AS MemberLastName, a.Mbr_ID AS MemberID, a.Contract_ID AS ContractID, a.Auth_Nbr AS AuthorizationorClaimNumber, a.Rcvd_Dt AS Datetherequestwasreceived FROM CMSUNIV_SRC_DEV_V.UM_AUTH a WHERE a.Btch_ID = {btch_id}</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV_FILELAND_$ENV_T</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>ODAG_DE_TABLE3_2022</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV_CORE_$ENV_T</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>ODAG_DE_TABLE3_2022</t>
-        </is>
-      </c>
-      <c r="K5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="N5" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="O5" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>ODAG3</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>SQLSERVER</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>cms_src_appeals_sqlsrv</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>SELECT m.FirstName AS MemberFirstName, m.LastName AS MemberLastName, m.MemberNumber AS MemberID, a.ContractId AS ContractID, a.AppealNumber AS AuthorizationorClaimNumber, CONVERT(varchar(10), a.ReceivedDate, 23) AS Datetherequestwasreceived FROM dbo.Appeal a JOIN dbo.Member m ON m.MemberKey = a.MemberKey WHERE a.Btch_ID = {btch_id}</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV_FILELAND_$ENV_T</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>ODAG_DE_TABLE3_2022</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>CMSUNIV_CORE_$ENV_T</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>ODAG_DE_TABLE3_2022</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="M6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-      <c r="N6" s="11" t="inlineStr">
-        <is>
-          <t>(default CURRENT_TIMESTAMP(6))</t>
-        </is>
-      </c>
-      <c r="O6" s="11" t="inlineStr">
-        <is>
-          <t>(default USER)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>